<commit_message>
Included judgemental analysis for components across time horizons
</commit_message>
<xml_diff>
--- a/3_Component_Results/PRIVCON/Data/ifo_err/ifo_qoq_errors_first_eval.xlsx
+++ b/3_Component_Results/PRIVCON/Data/ifo_err/ifo_qoq_errors_first_eval.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>Q0</t>
   </si>
@@ -200,6 +200,9 @@
   </si>
   <si>
     <t>2025-08-22 00:00:00_diff</t>
+  </si>
+  <si>
+    <t>2025-11-25 00:00:00_diff</t>
   </si>
 </sst>
 </file>
@@ -557,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -1801,6 +1804,9 @@
       <c r="I45">
         <v>0.2452723979283746</v>
       </c>
+      <c r="J45">
+        <v>0.4551464291630793</v>
+      </c>
     </row>
     <row r="46" spans="1:11">
       <c r="A46" s="1" t="s">
@@ -1827,6 +1833,9 @@
       <c r="H46">
         <v>0.3452723979283974</v>
       </c>
+      <c r="I46">
+        <v>0.5551464291630595</v>
+      </c>
     </row>
     <row r="47" spans="1:11">
       <c r="A47" s="1" t="s">
@@ -1850,6 +1859,9 @@
       <c r="G47">
         <v>0.3452723979283974</v>
       </c>
+      <c r="H47">
+        <v>0.5551464291630595</v>
+      </c>
     </row>
     <row r="48" spans="1:11">
       <c r="A48" s="1" t="s">
@@ -1870,8 +1882,11 @@
       <c r="F48">
         <v>0.505272397928394</v>
       </c>
-    </row>
-    <row r="49" spans="1:5">
+      <c r="G48">
+        <v>0.7551464191630828</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
       <c r="A49" s="1" t="s">
         <v>57</v>
       </c>
@@ -1887,8 +1902,11 @@
       <c r="E49">
         <v>0.545272397928386</v>
       </c>
-    </row>
-    <row r="50" spans="1:5">
+      <c r="F49">
+        <v>0.7551464291630623</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
       <c r="A50" s="1" t="s">
         <v>58</v>
       </c>
@@ -1901,8 +1919,11 @@
       <c r="D50">
         <v>0.2052723979283826</v>
       </c>
-    </row>
-    <row r="51" spans="1:5">
+      <c r="E50">
+        <v>0.4351464291630833</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
       <c r="A51" s="1" t="s">
         <v>59</v>
       </c>
@@ -1912,18 +1933,32 @@
       <c r="C51">
         <v>0.1852723979283866</v>
       </c>
-    </row>
-    <row r="52" spans="1:5">
+      <c r="D51">
+        <v>0.4851464291630663</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
       <c r="A52" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B52">
         <v>0.1452758398526868</v>
       </c>
-    </row>
-    <row r="53" spans="1:5">
+      <c r="C52">
+        <v>0.3551464291630708</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
       <c r="A53" s="1" t="s">
         <v>61</v>
+      </c>
+      <c r="B53">
+        <v>0.2951464291630685</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="1" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>